<commit_message>
Red causal 3N: movimiento ~8x mas lento y cero fotos (nodos con icono, sin imagenes)
</commit_message>
<xml_diff>
--- a/datos/red-causal-3n.xlsx
+++ b/datos/red-causal-3n.xlsx
@@ -1211,11 +1211,7 @@
           <t>Guion del grupo; UAESP</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>./assets/cx_bacterias.png</t>
-        </is>
-      </c>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
         <v>4.627</v>
       </c>
@@ -1419,11 +1415,7 @@
           <t>PMA El Burro (SDA); guion del grupo</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>./assets/foto_humedal.png</t>
-        </is>
-      </c>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
         <v>4.6396</v>
       </c>
@@ -1491,11 +1483,7 @@
           <t>PMA Techo (SDA); guion del grupo</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>./assets/inat_juncal.png</t>
-        </is>
-      </c>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
         <v>4.6305</v>
       </c>
@@ -1563,11 +1551,7 @@
           <t>PMA La Vaca (SDA); guion del grupo</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>./assets/inat_lenteja.png</t>
-        </is>
-      </c>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>4.624</v>
       </c>
@@ -1839,11 +1823,7 @@
           <t>Guion del grupo</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>./assets/cx_lixiviados.png</t>
-        </is>
-      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
         <v>4.633</v>
       </c>
@@ -2183,11 +2163,7 @@
           <t>Guion del grupo</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>./assets/cx_nutrientes.png</t>
-        </is>
-      </c>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
         <v>4.6289</v>
       </c>

</xml_diff>